<commit_message>
feat: add actions count
</commit_message>
<xml_diff>
--- a/external_files/tables/Estados.xlsx
+++ b/external_files/tables/Estados.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t xml:space="preserve">AC</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">AP</t>
   </si>
   <si>
-    <t xml:space="preserve">Amapá</t>
+    <t xml:space="preserve">Amapa</t>
   </si>
   <si>
     <t xml:space="preserve">AM</t>
@@ -55,15 +55,12 @@
     <t xml:space="preserve">CE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ceará</t>
+    <t xml:space="preserve">Distrito Federal</t>
   </si>
   <si>
     <t xml:space="preserve">DF</t>
   </si>
   <si>
-    <t xml:space="preserve">Distrito Federal</t>
-  </si>
-  <si>
     <t xml:space="preserve">ES</t>
   </si>
   <si>
@@ -73,13 +70,13 @@
     <t xml:space="preserve">GO</t>
   </si>
   <si>
-    <t xml:space="preserve">Goiás</t>
+    <t xml:space="preserve">Goias</t>
   </si>
   <si>
     <t xml:space="preserve">MA</t>
   </si>
   <si>
-    <t xml:space="preserve">Maranhão</t>
+    <t xml:space="preserve">Maranhao</t>
   </si>
   <si>
     <t xml:space="preserve">MT</t>
@@ -103,19 +100,19 @@
     <t xml:space="preserve">PA</t>
   </si>
   <si>
-    <t xml:space="preserve">Pará</t>
+    <t xml:space="preserve">Para</t>
   </si>
   <si>
     <t xml:space="preserve">PB</t>
   </si>
   <si>
-    <t xml:space="preserve">Paraíba</t>
+    <t xml:space="preserve">Paraiba</t>
   </si>
   <si>
     <t xml:space="preserve">PR</t>
   </si>
   <si>
-    <t xml:space="preserve">Paraná</t>
+    <t xml:space="preserve">Parana</t>
   </si>
   <si>
     <t xml:space="preserve">PE</t>
@@ -127,7 +124,7 @@
     <t xml:space="preserve">PI</t>
   </si>
   <si>
-    <t xml:space="preserve">Piauí</t>
+    <t xml:space="preserve">Piaui</t>
   </si>
   <si>
     <t xml:space="preserve">RJ</t>
@@ -151,7 +148,7 @@
     <t xml:space="preserve">RO</t>
   </si>
   <si>
-    <t xml:space="preserve">Rondônia</t>
+    <t xml:space="preserve">Rondonia</t>
   </si>
   <si>
     <t xml:space="preserve">RR</t>
@@ -169,7 +166,7 @@
     <t xml:space="preserve">SP</t>
   </si>
   <si>
-    <t xml:space="preserve">São Paulo</t>
+    <t xml:space="preserve">Sao Paulo</t>
   </si>
   <si>
     <t xml:space="preserve">SE</t>
@@ -462,8 +459,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -737,223 +738,223 @@
   <dimension ref="A1:B27"/>
   <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12.15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="0" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="0" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="0" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="0" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="0" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="0" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="0" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="0" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="0" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="0" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="0" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="0" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="0" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="0" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="0" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="0" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="0" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B27" s="0" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>